<commit_message>
🏠 Scan: 2026-08-12 15:38 UTC
</commit_message>
<xml_diff>
--- a/data/szperacz_mieszkaniowy.xlsx
+++ b/data/szperacz_mieszkaniowy.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q122"/>
+  <dimension ref="A1:Q123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3353,6 +3353,29 @@
         <v>-756</v>
       </c>
       <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>anomaly_detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>15:36</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D123" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
         <is>
           <t>anomaly_detected</t>
         </is>
@@ -29519,10 +29542,10 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>756</v>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>-756</v>
+        <v>0</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -29531,7 +29554,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 08:22</t>
+          <t>2026-08-12 15:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🏠 Scan: 2026-08-12 17:34 UTC
</commit_message>
<xml_diff>
--- a/data/szperacz_mieszkaniowy.xlsx
+++ b/data/szperacz_mieszkaniowy.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q123"/>
+  <dimension ref="A1:Q124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3376,6 +3376,29 @@
         <v>0</v>
       </c>
       <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>anomaly_detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D124" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
         <is>
           <t>anomaly_detected</t>
         </is>
@@ -29554,7 +29577,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 15:36</t>
+          <t>2026-08-12 17:33</t>
         </is>
       </c>
     </row>

</xml_diff>